<commit_message>
Fill in the CRM with the MX results from the Actions run
Verified via the crm-mx-check workflow (run 32042127872): 1 lead on Microsoft
365 (grade A), 5 on other providers (B), 5 discarded (Google Workspace, no MX
published, or no domain of their own). Rows now carry a concrete next action
instead of "verificar MX".

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Qv8xRzqfeVCABsZZa8kBCp
</commit_message>
<xml_diff>
--- a/docs/crm/Collectionat-CRM.xlsx
+++ b/docs/crm/Collectionat-CRM.xlsx
@@ -613,8 +613,16 @@
           <t>menacho.com.ar</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>sin MX</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
@@ -624,15 +632,19 @@
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>nuevo</t>
+          <t>verificado</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>verificar MX y tamaño</t>
+          <t>revisar: el dominio no publica MX, el mail puede estar en otro dominio</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr"/>
@@ -678,8 +690,16 @@
           <t>dacal.com.ar</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Google Workspace</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr">
         <is>
@@ -689,15 +709,19 @@
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>nuevo</t>
+          <t>verificado</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>verificar MX y tamaño</t>
+          <t>descartar: Google Workspace</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr"/>
@@ -743,8 +767,16 @@
           <t>jjyacoub.com.ar</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Google Workspace</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr">
         <is>
@@ -754,15 +786,19 @@
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>nuevo</t>
+          <t>verificado</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>verificar MX y tamaño</t>
+          <t>descartar: Google Workspace</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr"/>
@@ -808,8 +844,16 @@
           <t>mirtalibera.com.ar</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>otro: mail.mirtalibera.com.ar</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr">
         <is>
@@ -819,15 +863,19 @@
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>nuevo</t>
+          <t>verificado</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>verificar MX y tamaño</t>
+          <t>verificar tamaño antes de invertir tiempo</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr"/>
@@ -873,8 +921,16 @@
           <t>rivaspropiedades.com.ar</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>otro: rivaspropiedades.com.ar</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr">
         <is>
@@ -884,15 +940,19 @@
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>nuevo</t>
+          <t>verificado</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>verificar MX y tamaño</t>
+          <t>verificar tamaño antes de invertir tiempo</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr"/>
@@ -938,8 +998,16 @@
           <t>wsyasociados.com.ar</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Hosting propio</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr">
         <is>
@@ -949,15 +1017,19 @@
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>nuevo</t>
+          <t>verificado</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>verificar MX y tamaño</t>
+          <t>verificar tamaño antes de invertir tiempo</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr"/>
@@ -1003,8 +1075,16 @@
           <t>rochayasoc.com</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Microsoft 365</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr">
         <is>
@@ -1014,15 +1094,19 @@
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>nuevo</t>
+          <t>verificado</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>verificar MX y tamaño</t>
+          <t>buscar al Socio Administrador en LinkedIn</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr"/>
@@ -1068,8 +1152,16 @@
           <t>escribania-ungaro.com</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>otro: mx.serviciodecorreo.es</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr">
         <is>
@@ -1079,15 +1171,19 @@
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>nuevo</t>
+          <t>verificado</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>verificar MX y tamaño</t>
+          <t>verificar tamaño antes de invertir tiempo</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr"/>
@@ -1133,8 +1229,16 @@
           <t>escribaniaocampofrontini.com</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>otro: mx.serviciodecorreo.es</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr">
         <is>
@@ -1144,15 +1248,19 @@
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>nuevo</t>
+          <t>verificado</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>verificar MX y tamaño</t>
+          <t>verificar tamaño antes de invertir tiempo</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr"/>
@@ -1198,8 +1306,16 @@
           <t>administracionlamberti.com</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>sin MX</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr">
         <is>
@@ -1209,15 +1325,19 @@
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>nuevo</t>
+          <t>verificado</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>verificar MX y tamaño</t>
+          <t>revisar: el dominio no publica MX, el mail puede estar en otro dominio</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr"/>
@@ -1259,8 +1379,16 @@
         </is>
       </c>
       <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>sin dominio propio</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr">
         <is>
@@ -1270,7 +1398,11 @@
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="O12" t="inlineStr">
         <is>
           <t>nuevo</t>
@@ -1278,7 +1410,7 @@
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>verificar MX y tamaño</t>
+          <t>descartar: sin dominio propio</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr"/>

</xml_diff>

<commit_message>
Fill in contact details scraped from the leads' own sites
From Actions run 32042955201: 76 of 104 leads now carry an email and 87 a phone
number, taken from what each company publishes on its own site. Extra addresses
and numbers go to the notes column; the 16 sites that publish nothing are marked
for a Maps/LinkedIn lookup instead of being left silently empty. Placeholder
addresses shipped with website templates (tu@email.com, correo@empresa.com) and
malformed numbers are filtered out.

Also corrects one entry: CABAPROP is CUCICBA's listing portal, not a real estate
agency, so it is marked as not a lead.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Qv8xRzqfeVCABsZZa8kBCp
</commit_message>
<xml_diff>
--- a/docs/crm/Collectionat-CRM.xlsx
+++ b/docs/crm/Collectionat-CRM.xlsx
@@ -630,8 +630,16 @@
         </is>
       </c>
       <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>info@menacho.com.ar</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>30714377392</t>
+        </is>
+      </c>
       <c r="N2" t="inlineStr">
         <is>
           <t>C</t>
@@ -655,7 +663,7 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>La mas grande de la region segun su propio sitio. Verificar si administra alquileres o solo venta.</t>
+          <t>La mas grande de la region segun su propio sitio. Verificar si administra alquileres o solo venta. | otros tel: 2214452470</t>
         </is>
       </c>
     </row>
@@ -732,7 +740,7 @@
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Venta y alquiler en La Plata y City Bell.</t>
+          <t>Venta y alquiler en La Plata y City Bell. | el sitio no publica datos de contacto: buscar por Google Maps o LinkedIn</t>
         </is>
       </c>
     </row>
@@ -785,7 +793,11 @@
       </c>
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>+5492215974522</t>
+        </is>
+      </c>
       <c r="N4" t="inlineStr">
         <is>
           <t>C</t>
@@ -809,7 +821,7 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>Sucursales en La Plata y City Bell.</t>
+          <t>Sucursales en La Plata y City Bell. | otros tel: 02215974522, 02214802091</t>
         </is>
       </c>
     </row>
@@ -861,8 +873,16 @@
         </is>
       </c>
       <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>info@mirtalibera.com.ar</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>02214519585</t>
+        </is>
+      </c>
       <c r="N5" t="inlineStr">
         <is>
           <t>B</t>
@@ -886,7 +906,7 @@
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>Mas de 40 años de trayectoria. Posible menos de 8 empleados: verificar filtro 1.</t>
+          <t>Mas de 40 años de trayectoria. Posible menos de 8 empleados: verificar filtro 1. | otros mails: basile.matias99@gmail.com</t>
         </is>
       </c>
     </row>
@@ -963,7 +983,7 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>Alquiler y venta.</t>
+          <t>Alquiler y venta. | el sitio no publica datos de contacto: buscar por Google Maps o LinkedIn</t>
         </is>
       </c>
     </row>
@@ -1015,8 +1035,16 @@
         </is>
       </c>
       <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>wsyasoc@gmail.com</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>5491123992570</t>
+        </is>
+      </c>
       <c r="N7" t="inlineStr">
         <is>
           <t>B</t>
@@ -1092,8 +1120,16 @@
         </is>
       </c>
       <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>estudiojuridico.rocha@hotmail.com</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>2213526308</t>
+        </is>
+      </c>
       <c r="N8" t="inlineStr">
         <is>
           <t>A</t>
@@ -1169,8 +1205,16 @@
         </is>
       </c>
       <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>scriungaro@yahoo.com</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>5492214635199</t>
+        </is>
+      </c>
       <c r="N9" t="inlineStr">
         <is>
           <t>B</t>
@@ -1194,7 +1238,7 @@
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>Verificar sede: el resultado de busqueda no confirma la ciudad.</t>
+          <t>Verificar sede: el resultado de busqueda no confirma la ciudad. | otros mails: spiroungaro@gmail.com, escriungaro@yahoo.com | otros tel: +542214229123</t>
         </is>
       </c>
     </row>
@@ -1246,8 +1290,16 @@
         </is>
       </c>
       <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>clfrontini@gmail.com</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>0221155381226</t>
+        </is>
+      </c>
       <c r="N10" t="inlineStr">
         <is>
           <t>B</t>
@@ -1271,7 +1323,7 @@
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>Calle 48 990, La Plata.</t>
+          <t>Calle 48 990, La Plata. | otros tel: 2216002293</t>
         </is>
       </c>
     </row>
@@ -1348,7 +1400,7 @@
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>Diagonal 74 Nº 1681. Miembro de la Camara de Administradores de La Plata.</t>
+          <t>Diagonal 74 Nº 1681. Miembro de la Camara de Administradores de La Plata. | el sitio no publica datos de contacto: buscar por Google Maps o LinkedIn</t>
         </is>
       </c>
     </row>
@@ -1396,8 +1448,16 @@
         </is>
       </c>
       <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>dr.luisbarbieratti@gmail.com</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>2236155464</t>
+        </is>
+      </c>
       <c r="N12" t="inlineStr">
         <is>
           <t>C</t>
@@ -1474,7 +1534,11 @@
       </c>
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>5491167494074</t>
+        </is>
+      </c>
       <c r="N13" t="inlineStr">
         <is>
           <t>B</t>
@@ -1498,7 +1562,7 @@
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>Oficinas en CABA, Lanús, Lomas de Zamora y Quilmes: estructura multi-sede.</t>
+          <t>Oficinas en CABA, Lanús, Lomas de Zamora y Quilmes: estructura multi-sede. | otros tel: 541167494074</t>
         </is>
       </c>
     </row>
@@ -1550,8 +1614,16 @@
         </is>
       </c>
       <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr"/>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>estudiodrarabia@gmail.com</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>5491123626037</t>
+        </is>
+      </c>
       <c r="N14" t="inlineStr">
         <is>
           <t>B</t>
@@ -1628,7 +1700,11 @@
       </c>
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>541161356329</t>
+        </is>
+      </c>
       <c r="N15" t="inlineStr">
         <is>
           <t>B</t>
@@ -1652,7 +1728,7 @@
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>30 años, zona sur y CABA.</t>
+          <t>30 años, zona sur y CABA. | otros tel: 541142981622, 541158001515</t>
         </is>
       </c>
     </row>
@@ -1705,7 +1781,11 @@
       </c>
       <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr"/>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>01148125500</t>
+        </is>
+      </c>
       <c r="N16" t="inlineStr">
         <is>
           <t>A</t>
@@ -1729,7 +1809,7 @@
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>Av. Santa Fe 1621, tres pisos: probablemente el más grande de la lista.</t>
+          <t>Av. Santa Fe 1621, tres pisos: probablemente el más grande de la lista. | el sitio no publica datos de contacto: buscar por Google Maps o LinkedIn | Teléfono tomado de directorios profesionales (Chambers, Abogados.com.ar), no del sitio: confirmar al llamar. El sitio no publica mail.</t>
         </is>
       </c>
     </row>
@@ -1781,8 +1861,16 @@
         </is>
       </c>
       <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr"/>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>marialaura19761@hotmail.com</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>+5491148065415</t>
+        </is>
+      </c>
       <c r="N17" t="inlineStr">
         <is>
           <t>B</t>
@@ -1806,7 +1894,7 @@
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>Morón, San Justo, Merlo, Castelar.</t>
+          <t>Morón, San Justo, Merlo, Castelar. | otros tel: +5491160436482</t>
         </is>
       </c>
     </row>
@@ -1883,7 +1971,7 @@
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>Morón. Sucesiones y jubilaciones.</t>
+          <t>Morón. Sucesiones y jubilaciones. | el sitio no publica datos de contacto: buscar por Google Maps o LinkedIn</t>
         </is>
       </c>
     </row>
@@ -1960,7 +2048,7 @@
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>Castelar. Además administra consorcios y propiedades: doble dolor documental.</t>
+          <t>Castelar. Además administra consorcios y propiedades: doble dolor documental. | el sitio no publica datos de contacto: buscar por Google Maps o LinkedIn</t>
         </is>
       </c>
     </row>
@@ -2012,8 +2100,16 @@
         </is>
       </c>
       <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr"/>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>drsobek@yahoo.com.ar</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>+5491160144702</t>
+        </is>
+      </c>
       <c r="N20" t="inlineStr">
         <is>
           <t>B</t>
@@ -2089,8 +2185,16 @@
         </is>
       </c>
       <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
-      <c r="M21" t="inlineStr"/>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>info@estudiojuridicomendez.com.ar</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>5491135831019</t>
+        </is>
+      </c>
       <c r="N21" t="inlineStr">
         <is>
           <t>B</t>
@@ -2166,8 +2270,16 @@
         </is>
       </c>
       <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr"/>
-      <c r="M22" t="inlineStr"/>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>mc@abogadodeaccidente.ar</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>541131693621</t>
+        </is>
+      </c>
       <c r="N22" t="inlineStr">
         <is>
           <t>B</t>
@@ -2191,7 +2303,7 @@
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>Laboral y daños. Quilmes, Berazategui, Varela.</t>
+          <t>Laboral y daños. Quilmes, Berazategui, Varela. | otros mails: dc@abogadodeaccidente.ar, estudioramosartigas@outlook.com</t>
         </is>
       </c>
     </row>
@@ -2243,8 +2355,16 @@
         </is>
       </c>
       <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr"/>
-      <c r="M23" t="inlineStr"/>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>estudiojuridicodrgerez@gmail.com</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>5491166394493</t>
+        </is>
+      </c>
       <c r="N23" t="inlineStr">
         <is>
           <t>B</t>
@@ -2320,8 +2440,16 @@
         </is>
       </c>
       <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr"/>
-      <c r="M24" t="inlineStr"/>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>info@gdtabogados.com</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>5491133166267</t>
+        </is>
+      </c>
       <c r="N24" t="inlineStr">
         <is>
           <t>C</t>
@@ -2398,7 +2526,11 @@
       </c>
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr"/>
-      <c r="M25" t="inlineStr"/>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>5491159499529</t>
+        </is>
+      </c>
       <c r="N25" t="inlineStr">
         <is>
           <t>B</t>
@@ -2422,7 +2554,7 @@
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>Sucesiones.</t>
+          <t>Sucesiones. | otros tel: 5491138928664</t>
         </is>
       </c>
     </row>
@@ -2474,8 +2606,16 @@
         </is>
       </c>
       <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr"/>
-      <c r="M26" t="inlineStr"/>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>info@vilarinoabogados.com.ar</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>541140646941</t>
+        </is>
+      </c>
       <c r="N26" t="inlineStr">
         <is>
           <t>B</t>
@@ -2499,7 +2639,7 @@
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>Familia y sucesiones.</t>
+          <t>Familia y sucesiones. | otros mails: vilarino.abogados@gmail.com</t>
         </is>
       </c>
     </row>
@@ -2551,8 +2691,16 @@
         </is>
       </c>
       <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr"/>
-      <c r="M27" t="inlineStr"/>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>consultas@abogadadesucesiones.com.ar</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>541148940054</t>
+        </is>
+      </c>
       <c r="N27" t="inlineStr">
         <is>
           <t>B</t>
@@ -2576,7 +2724,7 @@
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>Sucesiones. Verificar tamaño: puede ser unipersonal.</t>
+          <t>Sucesiones. Verificar tamaño: puede ser unipersonal. | otros mails: estudiolasia@gmail.com | otros tel: 1131184958</t>
         </is>
       </c>
     </row>
@@ -2628,8 +2776,16 @@
         </is>
       </c>
       <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr"/>
-      <c r="M28" t="inlineStr"/>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>info@gdtabogados.com</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>5491133166267</t>
+        </is>
+      </c>
       <c r="N28" t="inlineStr">
         <is>
           <t>C</t>
@@ -2705,8 +2861,16 @@
         </is>
       </c>
       <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr"/>
-      <c r="M29" t="inlineStr"/>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>nt@ntabogados.com.ar</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>5491128788270</t>
+        </is>
+      </c>
       <c r="N29" t="inlineStr">
         <is>
           <t>C</t>
@@ -2782,8 +2946,16 @@
         </is>
       </c>
       <c r="K30" t="inlineStr"/>
-      <c r="L30" t="inlineStr"/>
-      <c r="M30" t="inlineStr"/>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>edificios@adm-consorcios.com.ar</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>5491123077816</t>
+        </is>
+      </c>
       <c r="N30" t="inlineStr">
         <is>
           <t>B</t>
@@ -2807,7 +2979,7 @@
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>Auditorías, relevamientos y asistencia legal.</t>
+          <t>Auditorías, relevamientos y asistencia legal. | otros tel: +5491150321413</t>
         </is>
       </c>
     </row>
@@ -2860,7 +3032,11 @@
       </c>
       <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr"/>
-      <c r="M31" t="inlineStr"/>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>+5491161475364</t>
+        </is>
+      </c>
       <c r="N31" t="inlineStr">
         <is>
           <t>C</t>
@@ -2936,8 +3112,16 @@
         </is>
       </c>
       <c r="K32" t="inlineStr"/>
-      <c r="L32" t="inlineStr"/>
-      <c r="M32" t="inlineStr"/>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>info@adsr.com.ar</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>5491163532857</t>
+        </is>
+      </c>
       <c r="N32" t="inlineStr">
         <is>
           <t>B</t>
@@ -3013,8 +3197,16 @@
         </is>
       </c>
       <c r="K33" t="inlineStr"/>
-      <c r="L33" t="inlineStr"/>
-      <c r="M33" t="inlineStr"/>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>cgr@cygba.com.ar</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>1159482000</t>
+        </is>
+      </c>
       <c r="N33" t="inlineStr">
         <is>
           <t>B</t>
@@ -3038,7 +3230,7 @@
       </c>
       <c r="S33" t="inlineStr">
         <is>
-          <t>Usa plataforma admFull: ya compraron software, verificar qué les falta.</t>
+          <t>Usa plataforma admFull: ya compraron software, verificar qué les falta. | otros mails: comercial@cygba.com.ar | otros tel: 0541143255337</t>
         </is>
       </c>
     </row>
@@ -3090,8 +3282,16 @@
         </is>
       </c>
       <c r="K34" t="inlineStr"/>
-      <c r="L34" t="inlineStr"/>
-      <c r="M34" t="inlineStr"/>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>contacto@administracionsasso.com.ar</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>01147869410</t>
+        </is>
+      </c>
       <c r="N34" t="inlineStr">
         <is>
           <t>B</t>
@@ -3115,7 +3315,7 @@
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>Complejos, torres, parques industriales: cartera grande.</t>
+          <t>Complejos, torres, parques industriales: cartera grande. | otros mails: sucursal.oeste@administracionsasso.com.ar, admsasso@gmail.com | otros tel: 01146353828</t>
         </is>
       </c>
     </row>
@@ -3167,8 +3367,16 @@
         </is>
       </c>
       <c r="K35" t="inlineStr"/>
-      <c r="L35" t="inlineStr"/>
-      <c r="M35" t="inlineStr"/>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>info@administracionesfromo.com</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>+541144311755</t>
+        </is>
+      </c>
       <c r="N35" t="inlineStr">
         <is>
           <t>B</t>
@@ -3192,7 +3400,7 @@
       </c>
       <c r="S35" t="inlineStr">
         <is>
-          <t>Gestión online de expensas.</t>
+          <t>Gestión online de expensas. | otros tel: +541115657871</t>
         </is>
       </c>
     </row>
@@ -3269,7 +3477,7 @@
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>Sistema Expensas Claras del GCBA.</t>
+          <t>Sistema Expensas Claras del GCBA. | el sitio no publica datos de contacto: buscar por Google Maps o LinkedIn</t>
         </is>
       </c>
     </row>
@@ -3321,8 +3529,16 @@
         </is>
       </c>
       <c r="K37" t="inlineStr"/>
-      <c r="L37" t="inlineStr"/>
-      <c r="M37" t="inlineStr"/>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>presupuestos@ramosestudio.com.ar</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>+5491139880664</t>
+        </is>
+      </c>
       <c r="N37" t="inlineStr">
         <is>
           <t>B</t>
@@ -3398,7 +3614,11 @@
         </is>
       </c>
       <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr"/>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>agconsorcios@gmail.com</t>
+        </is>
+      </c>
       <c r="M38" t="inlineStr"/>
       <c r="N38" t="inlineStr">
         <is>
@@ -3475,8 +3695,16 @@
         </is>
       </c>
       <c r="K39" t="inlineStr"/>
-      <c r="L39" t="inlineStr"/>
-      <c r="M39" t="inlineStr"/>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>consorcios@ezentya.com.ar</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>1140447900</t>
+        </is>
+      </c>
       <c r="N39" t="inlineStr">
         <is>
           <t>B</t>
@@ -3577,7 +3805,7 @@
       </c>
       <c r="S40" t="inlineStr">
         <is>
-          <t>Olivos, Vicente López, Martínez, San Isidro.</t>
+          <t>Olivos, Vicente López, Martínez, San Isidro. | el sitio no publica datos de contacto: buscar por Google Maps o LinkedIn</t>
         </is>
       </c>
     </row>
@@ -3629,8 +3857,16 @@
         </is>
       </c>
       <c r="K41" t="inlineStr"/>
-      <c r="L41" t="inlineStr"/>
-      <c r="M41" t="inlineStr"/>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>gybadm@gmail.com</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>5491164637887</t>
+        </is>
+      </c>
       <c r="N41" t="inlineStr">
         <is>
           <t>C</t>
@@ -3654,7 +3890,7 @@
       </c>
       <c r="S41" t="inlineStr">
         <is>
-          <t>Vicente López, La Lucila, Martínez, San Isidro.</t>
+          <t>Vicente López, La Lucila, Martínez, San Isidro. | otros tel: 47006492</t>
         </is>
       </c>
     </row>
@@ -3706,8 +3942,16 @@
         </is>
       </c>
       <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr"/>
-      <c r="M42" t="inlineStr"/>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>info@estudiodachamorro.com.ar</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>+5491158495257</t>
+        </is>
+      </c>
       <c r="N42" t="inlineStr">
         <is>
           <t>B</t>
@@ -3731,7 +3975,7 @@
       </c>
       <c r="S42" t="inlineStr">
         <is>
-          <t>Contable + consorcios en Ramos Mejía y Haedo.</t>
+          <t>Contable + consorcios en Ramos Mejía y Haedo. | otros mails: infohaedo@estudiodachamorro.com.ar | otros tel: +5491132275570</t>
         </is>
       </c>
     </row>
@@ -3783,8 +4027,16 @@
         </is>
       </c>
       <c r="K43" t="inlineStr"/>
-      <c r="L43" t="inlineStr"/>
-      <c r="M43" t="inlineStr"/>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>info@smestudiocontable.com.ar</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>+541149778503</t>
+        </is>
+      </c>
       <c r="N43" t="inlineStr">
         <is>
           <t>B</t>
@@ -3808,7 +4060,7 @@
       </c>
       <c r="S43" t="inlineStr">
         <is>
-          <t>Contable con área de consorcios.</t>
+          <t>Contable con área de consorcios. | otros tel: +541135424060</t>
         </is>
       </c>
     </row>
@@ -3861,7 +4113,11 @@
       </c>
       <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr"/>
-      <c r="M44" t="inlineStr"/>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>+541155645320</t>
+        </is>
+      </c>
       <c r="N44" t="inlineStr">
         <is>
           <t>B</t>
@@ -3937,8 +4193,16 @@
         </is>
       </c>
       <c r="K45" t="inlineStr"/>
-      <c r="L45" t="inlineStr"/>
-      <c r="M45" t="inlineStr"/>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>hola@administrador-de-consorcios.com.ar</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>1161712616</t>
+        </is>
+      </c>
       <c r="N45" t="inlineStr">
         <is>
           <t>B</t>
@@ -3962,7 +4226,7 @@
       </c>
       <c r="S45" t="inlineStr">
         <is>
-          <t>Cubre CABA y AMBA.</t>
+          <t>Cubre CABA y AMBA. | otros mails: administracion@zanotticonsorcios.com.ar</t>
         </is>
       </c>
     </row>
@@ -4014,8 +4278,16 @@
         </is>
       </c>
       <c r="K46" t="inlineStr"/>
-      <c r="L46" t="inlineStr"/>
-      <c r="M46" t="inlineStr"/>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>info@brick.com.ar</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>5491153292035</t>
+        </is>
+      </c>
       <c r="N46" t="inlineStr">
         <is>
           <t>C</t>
@@ -4039,7 +4311,7 @@
       </c>
       <c r="S46" t="inlineStr">
         <is>
-          <t>CABA, zona norte y sur. Administración de alquileres.</t>
+          <t>CABA, zona norte y sur. Administración de alquileres. | otros tel: 5491130017060</t>
         </is>
       </c>
     </row>
@@ -4091,8 +4363,16 @@
         </is>
       </c>
       <c r="K47" t="inlineStr"/>
-      <c r="L47" t="inlineStr"/>
-      <c r="M47" t="inlineStr"/>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>info@administracioncaba.com.ar</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>5491176090964</t>
+        </is>
+      </c>
       <c r="N47" t="inlineStr">
         <is>
           <t>B</t>
@@ -4116,7 +4396,7 @@
       </c>
       <c r="S47" t="inlineStr">
         <is>
-          <t>Especializada en administración de locaciones: fit alto.</t>
+          <t>Especializada en administración de locaciones: fit alto. | otros tel: 5491126379317</t>
         </is>
       </c>
     </row>
@@ -4168,8 +4448,16 @@
         </is>
       </c>
       <c r="K48" t="inlineStr"/>
-      <c r="L48" t="inlineStr"/>
-      <c r="M48" t="inlineStr"/>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>info@theunionpropiedades.com</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>541149629888</t>
+        </is>
+      </c>
       <c r="N48" t="inlineStr">
         <is>
           <t>B</t>
@@ -4193,7 +4481,7 @@
       </c>
       <c r="S48" t="inlineStr">
         <is>
-          <t>Compra, venta y alquiler.</t>
+          <t>Compra, venta y alquiler. | otros tel: 541130261973</t>
         </is>
       </c>
     </row>
@@ -4245,8 +4533,16 @@
         </is>
       </c>
       <c r="K49" t="inlineStr"/>
-      <c r="L49" t="inlineStr"/>
-      <c r="M49" t="inlineStr"/>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>info@atbuenosaires.com</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>5491167227457</t>
+        </is>
+      </c>
       <c r="N49" t="inlineStr">
         <is>
           <t>C</t>
@@ -4326,17 +4622,17 @@
       <c r="M50" t="inlineStr"/>
       <c r="N50" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>verificado</t>
+          <t>descartado</t>
         </is>
       </c>
       <c r="P50" t="inlineStr">
         <is>
-          <t>PRIORIDAD: buscar al Gerente de Administración en LinkedIn</t>
+          <t>descartar: no es empresa</t>
         </is>
       </c>
       <c r="Q50" t="inlineStr"/>
@@ -4347,7 +4643,7 @@
       </c>
       <c r="S50" t="inlineStr">
         <is>
-          <t>Propiedades y emprendimientos.</t>
+          <t>NO ES LEAD: es el portal inmobiliario de CUCICBA (el colegio de corredores), no una inmobiliaria. Lo dejo en la base para que no se vuelva a cargar por error. Su listado de inmobiliarias socias sí sirve como fuente de leads nuevos.</t>
         </is>
       </c>
     </row>
@@ -4399,8 +4695,16 @@
         </is>
       </c>
       <c r="K51" t="inlineStr"/>
-      <c r="L51" t="inlineStr"/>
-      <c r="M51" t="inlineStr"/>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>recoleta@izr.com.ar</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>01152791001</t>
+        </is>
+      </c>
       <c r="N51" t="inlineStr">
         <is>
           <t>C</t>
@@ -4424,7 +4728,7 @@
       </c>
       <c r="S51" t="inlineStr">
         <is>
-          <t>+40 años. Vicente López, Olivos, San Isidro.</t>
+          <t>+40 años. Vicente López, Olivos, San Isidro. | otros mails: tasaciones@izr.com.ar | otros tel: 5491138309311</t>
         </is>
       </c>
     </row>
@@ -4501,7 +4805,7 @@
       </c>
       <c r="S52" t="inlineStr">
         <is>
-          <t>Más de 50 años en zona norte.</t>
+          <t>Más de 50 años en zona norte. | el sitio no publica datos de contacto: buscar por Google Maps o LinkedIn</t>
         </is>
       </c>
     </row>
@@ -4553,8 +4857,16 @@
         </is>
       </c>
       <c r="K53" t="inlineStr"/>
-      <c r="L53" t="inlineStr"/>
-      <c r="M53" t="inlineStr"/>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>encontacto@torresprop.com</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>5491131091200</t>
+        </is>
+      </c>
       <c r="N53" t="inlineStr">
         <is>
           <t>C</t>
@@ -4630,8 +4942,16 @@
         </is>
       </c>
       <c r="K54" t="inlineStr"/>
-      <c r="L54" t="inlineStr"/>
-      <c r="M54" t="inlineStr"/>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>info@veninipropiedades.com</t>
+        </is>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>541152210196</t>
+        </is>
+      </c>
       <c r="N54" t="inlineStr">
         <is>
           <t>B</t>
@@ -4707,8 +5027,16 @@
         </is>
       </c>
       <c r="K55" t="inlineStr"/>
-      <c r="L55" t="inlineStr"/>
-      <c r="M55" t="inlineStr"/>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>inmobiliariaiacono@gmail.com</t>
+        </is>
+      </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>5491138500812</t>
+        </is>
+      </c>
       <c r="N55" t="inlineStr">
         <is>
           <t>C</t>
@@ -4784,8 +5112,16 @@
         </is>
       </c>
       <c r="K56" t="inlineStr"/>
-      <c r="L56" t="inlineStr"/>
-      <c r="M56" t="inlineStr"/>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>joforciniti@hotmail.com</t>
+        </is>
+      </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>+5491158208040</t>
+        </is>
+      </c>
       <c r="N56" t="inlineStr">
         <is>
           <t>B</t>
@@ -4809,7 +5145,7 @@
       </c>
       <c r="S56" t="inlineStr">
         <is>
-          <t>Quilmes.</t>
+          <t>Quilmes. | otros tel: 42104555</t>
         </is>
       </c>
     </row>
@@ -4886,7 +5222,7 @@
       </c>
       <c r="S57" t="inlineStr">
         <is>
-          <t>Quilmes.</t>
+          <t>Quilmes. | el sitio no publica datos de contacto: buscar por Google Maps o LinkedIn</t>
         </is>
       </c>
     </row>
@@ -4963,7 +5299,7 @@
       </c>
       <c r="S58" t="inlineStr">
         <is>
-          <t>Alquiler y venta.</t>
+          <t>Alquiler y venta. | el sitio no publica datos de contacto: buscar por Google Maps o LinkedIn</t>
         </is>
       </c>
     </row>
@@ -5015,8 +5351,16 @@
         </is>
       </c>
       <c r="K59" t="inlineStr"/>
-      <c r="L59" t="inlineStr"/>
-      <c r="M59" t="inlineStr"/>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>inmobiliaria.alsina@gmail.com</t>
+        </is>
+      </c>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>5491142548838</t>
+        </is>
+      </c>
       <c r="N59" t="inlineStr">
         <is>
           <t>B</t>
@@ -5092,8 +5436,16 @@
         </is>
       </c>
       <c r="K60" t="inlineStr"/>
-      <c r="L60" t="inlineStr"/>
-      <c r="M60" t="inlineStr"/>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>urquizapropiedades2000@gmail.com</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>+5491164660770</t>
+        </is>
+      </c>
       <c r="N60" t="inlineStr">
         <is>
           <t>B</t>
@@ -5169,8 +5521,16 @@
         </is>
       </c>
       <c r="K61" t="inlineStr"/>
-      <c r="L61" t="inlineStr"/>
-      <c r="M61" t="inlineStr"/>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>info@carlosmilani.com</t>
+        </is>
+      </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>5491157956424</t>
+        </is>
+      </c>
       <c r="N61" t="inlineStr">
         <is>
           <t>B</t>
@@ -5194,7 +5554,7 @@
       </c>
       <c r="S61" t="inlineStr">
         <is>
-          <t>Morón, Ramos Mejía, Ituzaingó.</t>
+          <t>Morón, Ramos Mejía, Ituzaingó. | otros tel: 1156569619</t>
         </is>
       </c>
     </row>
@@ -5246,8 +5606,16 @@
         </is>
       </c>
       <c r="K62" t="inlineStr"/>
-      <c r="L62" t="inlineStr"/>
-      <c r="M62" t="inlineStr"/>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>vita@remax.com.ar</t>
+        </is>
+      </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>44893929</t>
+        </is>
+      </c>
       <c r="N62" t="inlineStr">
         <is>
           <t>C</t>
@@ -5324,7 +5692,11 @@
       </c>
       <c r="K63" t="inlineStr"/>
       <c r="L63" t="inlineStr"/>
-      <c r="M63" t="inlineStr"/>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>3495585122</t>
+        </is>
+      </c>
       <c r="N63" t="inlineStr">
         <is>
           <t>B</t>
@@ -5348,7 +5720,7 @@
       </c>
       <c r="S63" t="inlineStr">
         <is>
-          <t>Morón.</t>
+          <t>Morón. | otros tel: 3469524233</t>
         </is>
       </c>
     </row>
@@ -5400,8 +5772,16 @@
         </is>
       </c>
       <c r="K64" t="inlineStr"/>
-      <c r="L64" t="inlineStr"/>
-      <c r="M64" t="inlineStr"/>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>info@sambrapropiedades.com.ar</t>
+        </is>
+      </c>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>01147869286</t>
+        </is>
+      </c>
       <c r="N64" t="inlineStr">
         <is>
           <t>B</t>
@@ -5425,7 +5805,7 @@
       </c>
       <c r="S64" t="inlineStr">
         <is>
-          <t>Belgrano, Caballito, Flores, Villa Urquiza. Administra propiedades.</t>
+          <t>Belgrano, Caballito, Flores, Villa Urquiza. Administra propiedades. | otros tel: 1137948907</t>
         </is>
       </c>
     </row>
@@ -5477,8 +5857,16 @@
         </is>
       </c>
       <c r="K65" t="inlineStr"/>
-      <c r="L65" t="inlineStr"/>
-      <c r="M65" t="inlineStr"/>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>cramer@dodorico.com</t>
+        </is>
+      </c>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>5491172873030</t>
+        </is>
+      </c>
       <c r="N65" t="inlineStr">
         <is>
           <t>B</t>
@@ -5502,7 +5890,7 @@
       </c>
       <c r="S65" t="inlineStr">
         <is>
-          <t>+40 años, varias sucursales en CABA.</t>
+          <t>+40 años, varias sucursales en CABA. | otros mails: alberdi@dodorico.com, laplata@dodorico.com | otros tel: 5491172873033</t>
         </is>
       </c>
     </row>
@@ -5579,7 +5967,7 @@
       </c>
       <c r="S66" t="inlineStr">
         <is>
-          <t>Caballito y Villa Urquiza.</t>
+          <t>Caballito y Villa Urquiza. | el sitio no publica datos de contacto: buscar por Google Maps o LinkedIn</t>
         </is>
       </c>
     </row>
@@ -5631,8 +6019,16 @@
         </is>
       </c>
       <c r="K67" t="inlineStr"/>
-      <c r="L67" t="inlineStr"/>
-      <c r="M67" t="inlineStr"/>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>info@urquiza.com.ar</t>
+        </is>
+      </c>
+      <c r="M67" t="inlineStr">
+        <is>
+          <t>2214802742</t>
+        </is>
+      </c>
       <c r="N67" t="inlineStr">
         <is>
           <t>C</t>
@@ -5656,7 +6052,7 @@
       </c>
       <c r="S67" t="inlineStr">
         <is>
-          <t>Desde 1982. City Bell, Gonnet, Villa Elisa.</t>
+          <t>Desde 1982. City Bell, Gonnet, Villa Elisa. | otros tel: 5492216682190</t>
         </is>
       </c>
     </row>
@@ -5708,8 +6104,16 @@
         </is>
       </c>
       <c r="K68" t="inlineStr"/>
-      <c r="L68" t="inlineStr"/>
-      <c r="M68" t="inlineStr"/>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>ventas@camiglia.com.ar</t>
+        </is>
+      </c>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>+542214365851</t>
+        </is>
+      </c>
       <c r="N68" t="inlineStr">
         <is>
           <t>B</t>
@@ -5733,7 +6137,7 @@
       </c>
       <c r="S68" t="inlineStr">
         <is>
-          <t>Gonnet y La Plata.</t>
+          <t>Gonnet y La Plata. | otros mails: camiglia@hotmail.com | otros tel: +542214710026</t>
         </is>
       </c>
     </row>
@@ -5785,8 +6189,16 @@
         </is>
       </c>
       <c r="K69" t="inlineStr"/>
-      <c r="L69" t="inlineStr"/>
-      <c r="M69" t="inlineStr"/>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>info@svyasociados.com</t>
+        </is>
+      </c>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>+541150328709</t>
+        </is>
+      </c>
       <c r="N69" t="inlineStr">
         <is>
           <t>C</t>
@@ -5810,7 +6222,7 @@
       </c>
       <c r="S69" t="inlineStr">
         <is>
-          <t>Jurídico-contable en Belgrano: doble vertical.</t>
+          <t>Jurídico-contable en Belgrano: doble vertical. | otros tel: 5491124538863</t>
         </is>
       </c>
     </row>
@@ -5862,8 +6274,16 @@
         </is>
       </c>
       <c r="K70" t="inlineStr"/>
-      <c r="L70" t="inlineStr"/>
-      <c r="M70" t="inlineStr"/>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>info@craiem.com.ar</t>
+        </is>
+      </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>+5491145611024</t>
+        </is>
+      </c>
       <c r="N70" t="inlineStr">
         <is>
           <t>C</t>
@@ -5939,8 +6359,16 @@
         </is>
       </c>
       <c r="K71" t="inlineStr"/>
-      <c r="L71" t="inlineStr"/>
-      <c r="M71" t="inlineStr"/>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>kevin@estudiosaied.com.ar</t>
+        </is>
+      </c>
+      <c r="M71" t="inlineStr">
+        <is>
+          <t>01120071465</t>
+        </is>
+      </c>
       <c r="N71" t="inlineStr">
         <is>
           <t>B</t>
@@ -5964,7 +6392,7 @@
       </c>
       <c r="S71" t="inlineStr">
         <is>
-          <t>Av. Nazca 890. PyMEs y unipersonales.</t>
+          <t>Av. Nazca 890. PyMEs y unipersonales. | otros tel: 01154022741</t>
         </is>
       </c>
     </row>
@@ -6016,8 +6444,16 @@
         </is>
       </c>
       <c r="K72" t="inlineStr"/>
-      <c r="L72" t="inlineStr"/>
-      <c r="M72" t="inlineStr"/>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>info@e-cont.com.ar</t>
+        </is>
+      </c>
+      <c r="M72" t="inlineStr">
+        <is>
+          <t>5491157023328</t>
+        </is>
+      </c>
       <c r="N72" t="inlineStr">
         <is>
           <t>C</t>
@@ -6093,8 +6529,16 @@
         </is>
       </c>
       <c r="K73" t="inlineStr"/>
-      <c r="L73" t="inlineStr"/>
-      <c r="M73" t="inlineStr"/>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>info@estudiocontablealwa.com.ar</t>
+        </is>
+      </c>
+      <c r="M73" t="inlineStr">
+        <is>
+          <t>5491164786951</t>
+        </is>
+      </c>
       <c r="N73" t="inlineStr">
         <is>
           <t>C</t>
@@ -6171,7 +6615,11 @@
       </c>
       <c r="K74" t="inlineStr"/>
       <c r="L74" t="inlineStr"/>
-      <c r="M74" t="inlineStr"/>
+      <c r="M74" t="inlineStr">
+        <is>
+          <t>5491160485050</t>
+        </is>
+      </c>
       <c r="N74" t="inlineStr">
         <is>
           <t>C</t>
@@ -6247,8 +6695,16 @@
         </is>
       </c>
       <c r="K75" t="inlineStr"/>
-      <c r="L75" t="inlineStr"/>
-      <c r="M75" t="inlineStr"/>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>info@estudiomc.com.ar</t>
+        </is>
+      </c>
+      <c r="M75" t="inlineStr">
+        <is>
+          <t>48407160</t>
+        </is>
+      </c>
       <c r="N75" t="inlineStr">
         <is>
           <t>B</t>
@@ -6324,8 +6780,16 @@
         </is>
       </c>
       <c r="K76" t="inlineStr"/>
-      <c r="L76" t="inlineStr"/>
-      <c r="M76" t="inlineStr"/>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>info@estudiopiacentini.com.ar</t>
+        </is>
+      </c>
+      <c r="M76" t="inlineStr">
+        <is>
+          <t>45853779</t>
+        </is>
+      </c>
       <c r="N76" t="inlineStr">
         <is>
           <t>B</t>
@@ -6349,7 +6813,7 @@
       </c>
       <c r="S76" t="inlineStr">
         <is>
-          <t>Villa del Parque.</t>
+          <t>Villa del Parque. | otros mails: atencionclientes@estudiopiacentini.com.ar | otros tel: 1551435065</t>
         </is>
       </c>
     </row>
@@ -6426,7 +6890,7 @@
       </c>
       <c r="S77" t="inlineStr">
         <is>
-          <t>San Isidro, Vicente López, Olivos.</t>
+          <t>San Isidro, Vicente López, Olivos. | el sitio no publica datos de contacto: buscar por Google Maps o LinkedIn</t>
         </is>
       </c>
     </row>
@@ -6478,8 +6942,16 @@
         </is>
       </c>
       <c r="K78" t="inlineStr"/>
-      <c r="L78" t="inlineStr"/>
-      <c r="M78" t="inlineStr"/>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>bokoestudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="M78" t="inlineStr">
+        <is>
+          <t>1168616903</t>
+        </is>
+      </c>
       <c r="N78" t="inlineStr">
         <is>
           <t>B</t>
@@ -6555,8 +7027,16 @@
         </is>
       </c>
       <c r="K79" t="inlineStr"/>
-      <c r="L79" t="inlineStr"/>
-      <c r="M79" t="inlineStr"/>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>consulta@estudiocontablenorte.com.ar</t>
+        </is>
+      </c>
+      <c r="M79" t="inlineStr">
+        <is>
+          <t>+5491167999289</t>
+        </is>
+      </c>
       <c r="N79" t="inlineStr">
         <is>
           <t>B</t>
@@ -6632,8 +7112,16 @@
         </is>
       </c>
       <c r="K80" t="inlineStr"/>
-      <c r="L80" t="inlineStr"/>
-      <c r="M80" t="inlineStr"/>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>info@moralesyasociados.com.ar</t>
+        </is>
+      </c>
+      <c r="M80" t="inlineStr">
+        <is>
+          <t>541144922027</t>
+        </is>
+      </c>
       <c r="N80" t="inlineStr">
         <is>
           <t>B</t>
@@ -6657,7 +7145,7 @@
       </c>
       <c r="S80" t="inlineStr">
         <is>
-          <t>Quilmes, Bernal, Lomas, La Plata. Cartera amplia: multiplicador.</t>
+          <t>Quilmes, Bernal, Lomas, La Plata. Cartera amplia: multiplicador. | otros tel: 541167625236</t>
         </is>
       </c>
     </row>
@@ -6709,8 +7197,16 @@
         </is>
       </c>
       <c r="K81" t="inlineStr"/>
-      <c r="L81" t="inlineStr"/>
-      <c r="M81" t="inlineStr"/>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>estudiozurano@gmail.com</t>
+        </is>
+      </c>
+      <c r="M81" t="inlineStr">
+        <is>
+          <t>01142880296</t>
+        </is>
+      </c>
       <c r="N81" t="inlineStr">
         <is>
           <t>B</t>
@@ -6734,7 +7230,7 @@
       </c>
       <c r="S81" t="inlineStr">
         <is>
-          <t>Lomas de Zamora, +20 años.</t>
+          <t>Lomas de Zamora, +20 años. | otros tel: 5491153852249</t>
         </is>
       </c>
     </row>
@@ -6786,8 +7282,16 @@
         </is>
       </c>
       <c r="K82" t="inlineStr"/>
-      <c r="L82" t="inlineStr"/>
-      <c r="M82" t="inlineStr"/>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>info@estudiocontablemm.com.ar</t>
+        </is>
+      </c>
+      <c r="M82" t="inlineStr">
+        <is>
+          <t>01159507280</t>
+        </is>
+      </c>
       <c r="N82" t="inlineStr">
         <is>
           <t>B</t>
@@ -6811,7 +7315,7 @@
       </c>
       <c r="S82" t="inlineStr">
         <is>
-          <t>Lomas de Zamora. Administración de PyMEs.</t>
+          <t>Lomas de Zamora. Administración de PyMEs. | otros mails: estudiocontablemascheroni@gmail.com | otros tel: 1171056527</t>
         </is>
       </c>
     </row>
@@ -6863,8 +7367,16 @@
         </is>
       </c>
       <c r="K83" t="inlineStr"/>
-      <c r="L83" t="inlineStr"/>
-      <c r="M83" t="inlineStr"/>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>info@estudiolomazzi.com</t>
+        </is>
+      </c>
+      <c r="M83" t="inlineStr">
+        <is>
+          <t>5491149472324</t>
+        </is>
+      </c>
       <c r="N83" t="inlineStr">
         <is>
           <t>B</t>
@@ -6888,7 +7400,7 @@
       </c>
       <c r="S83" t="inlineStr">
         <is>
-          <t>Quilmes. Especialistas en PyMEs.</t>
+          <t>Quilmes. Especialistas en PyMEs. | otros tel: 08102680116</t>
         </is>
       </c>
     </row>
@@ -6940,8 +7452,16 @@
         </is>
       </c>
       <c r="K84" t="inlineStr"/>
-      <c r="L84" t="inlineStr"/>
-      <c r="M84" t="inlineStr"/>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>info@asociadoscontables.com.ar</t>
+        </is>
+      </c>
+      <c r="M84" t="inlineStr">
+        <is>
+          <t>541124013444</t>
+        </is>
+      </c>
       <c r="N84" t="inlineStr">
         <is>
           <t>B</t>
@@ -6965,7 +7485,7 @@
       </c>
       <c r="S84" t="inlineStr">
         <is>
-          <t>Tres generaciones. La Plata, Berisso, Ensenada.</t>
+          <t>Tres generaciones. La Plata, Berisso, Ensenada. | otros tel: +5491531978441</t>
         </is>
       </c>
     </row>
@@ -7018,7 +7538,11 @@
       </c>
       <c r="K85" t="inlineStr"/>
       <c r="L85" t="inlineStr"/>
-      <c r="M85" t="inlineStr"/>
+      <c r="M85" t="inlineStr">
+        <is>
+          <t>2216258936</t>
+        </is>
+      </c>
       <c r="N85" t="inlineStr">
         <is>
           <t>B</t>
@@ -7095,7 +7619,11 @@
       </c>
       <c r="K86" t="inlineStr"/>
       <c r="L86" t="inlineStr"/>
-      <c r="M86" t="inlineStr"/>
+      <c r="M86" t="inlineStr">
+        <is>
+          <t>542214548808</t>
+        </is>
+      </c>
       <c r="N86" t="inlineStr">
         <is>
           <t>C</t>
@@ -7171,8 +7699,16 @@
         </is>
       </c>
       <c r="K87" t="inlineStr"/>
-      <c r="L87" t="inlineStr"/>
-      <c r="M87" t="inlineStr"/>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>contacto@escribaniahda.com.ar</t>
+        </is>
+      </c>
+      <c r="M87" t="inlineStr">
+        <is>
+          <t>+5491152632005</t>
+        </is>
+      </c>
       <c r="N87" t="inlineStr">
         <is>
           <t>C</t>
@@ -7248,8 +7784,16 @@
         </is>
       </c>
       <c r="K88" t="inlineStr"/>
-      <c r="L88" t="inlineStr"/>
-      <c r="M88" t="inlineStr"/>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>escribaniasalierno@gmail.com</t>
+        </is>
+      </c>
+      <c r="M88" t="inlineStr">
+        <is>
+          <t>1125371585</t>
+        </is>
+      </c>
       <c r="N88" t="inlineStr">
         <is>
           <t>B</t>
@@ -7325,8 +7869,16 @@
         </is>
       </c>
       <c r="K89" t="inlineStr"/>
-      <c r="L89" t="inlineStr"/>
-      <c r="M89" t="inlineStr"/>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>escribania@escribaniadamore.com.ar</t>
+        </is>
+      </c>
+      <c r="M89" t="inlineStr">
+        <is>
+          <t>+5491155857475</t>
+        </is>
+      </c>
       <c r="N89" t="inlineStr">
         <is>
           <t>B</t>
@@ -7350,7 +7902,7 @@
       </c>
       <c r="S89" t="inlineStr">
         <is>
-          <t>Lomas de Zamora, 70 años de historia.</t>
+          <t>Lomas de Zamora, 70 años de historia. | otros tel: +5491124639928</t>
         </is>
       </c>
     </row>
@@ -7402,8 +7954,16 @@
         </is>
       </c>
       <c r="K90" t="inlineStr"/>
-      <c r="L90" t="inlineStr"/>
-      <c r="M90" t="inlineStr"/>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>ventas@diemar.com.ar</t>
+        </is>
+      </c>
+      <c r="M90" t="inlineStr">
+        <is>
+          <t>5491141408397</t>
+        </is>
+      </c>
       <c r="N90" t="inlineStr">
         <is>
           <t>C</t>
@@ -7479,8 +8039,16 @@
         </is>
       </c>
       <c r="K91" t="inlineStr"/>
-      <c r="L91" t="inlineStr"/>
-      <c r="M91" t="inlineStr"/>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>distribuidorahomepoint@gmail.com</t>
+        </is>
+      </c>
+      <c r="M91" t="inlineStr">
+        <is>
+          <t>+5491121891006</t>
+        </is>
+      </c>
       <c r="N91" t="inlineStr">
         <is>
           <t>C</t>
@@ -7504,7 +8072,7 @@
       </c>
       <c r="S91" t="inlineStr">
         <is>
-          <t>Munro. Familiar.</t>
+          <t>Munro. Familiar. | otros tel: +5491176460030</t>
         </is>
       </c>
     </row>
@@ -7556,8 +8124,16 @@
         </is>
       </c>
       <c r="K92" t="inlineStr"/>
-      <c r="L92" t="inlineStr"/>
-      <c r="M92" t="inlineStr"/>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>ventas@masivos.com</t>
+        </is>
+      </c>
+      <c r="M92" t="inlineStr">
+        <is>
+          <t>5491141877697</t>
+        </is>
+      </c>
       <c r="N92" t="inlineStr">
         <is>
           <t>B</t>
@@ -7581,7 +8157,7 @@
       </c>
       <c r="S92" t="inlineStr">
         <is>
-          <t>Devoto. Comestibles, limpieza, kiosco.</t>
+          <t>Devoto. Comestibles, limpieza, kiosco. | otros tel: 1146862382</t>
         </is>
       </c>
     </row>
@@ -7633,8 +8209,16 @@
         </is>
       </c>
       <c r="K93" t="inlineStr"/>
-      <c r="L93" t="inlineStr"/>
-      <c r="M93" t="inlineStr"/>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>info@buenosaireslimpieza.com</t>
+        </is>
+      </c>
+      <c r="M93" t="inlineStr">
+        <is>
+          <t>5491159690884</t>
+        </is>
+      </c>
       <c r="N93" t="inlineStr">
         <is>
           <t>B</t>
@@ -7658,7 +8242,7 @@
       </c>
       <c r="S93" t="inlineStr">
         <is>
-          <t>Familiar, +70 años.</t>
+          <t>Familiar, +70 años. | otros mails: pedidos@buenosaireslimpieza.com.ar</t>
         </is>
       </c>
     </row>
@@ -7710,8 +8294,16 @@
         </is>
       </c>
       <c r="K94" t="inlineStr"/>
-      <c r="L94" t="inlineStr"/>
-      <c r="M94" t="inlineStr"/>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>contacto@el-sembrador.com.ar</t>
+        </is>
+      </c>
+      <c r="M94" t="inlineStr">
+        <is>
+          <t>+542604815957</t>
+        </is>
+      </c>
       <c r="N94" t="inlineStr">
         <is>
           <t>B</t>
@@ -7735,7 +8327,7 @@
       </c>
       <c r="S94" t="inlineStr">
         <is>
-          <t>Alimentos saludables.</t>
+          <t>Alimentos saludables. | otros tel: +542604039060</t>
         </is>
       </c>
     </row>
@@ -7787,8 +8379,16 @@
         </is>
       </c>
       <c r="K95" t="inlineStr"/>
-      <c r="L95" t="inlineStr"/>
-      <c r="M95" t="inlineStr"/>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>ventas@frigorificosada.com.ar</t>
+        </is>
+      </c>
+      <c r="M95" t="inlineStr">
+        <is>
+          <t>+542326456479</t>
+        </is>
+      </c>
       <c r="N95" t="inlineStr">
         <is>
           <t>B</t>
@@ -7812,7 +8412,7 @@
       </c>
       <c r="S95" t="inlineStr">
         <is>
-          <t>Ojo: frigorífico puede ser industria con ERP propio, no distribución pura.</t>
+          <t>Ojo: frigorífico puede ser industria con ERP propio, no distribución pura. | otros mails: rrhh@frigorificosada.com.ar | otros tel: 5492326464720</t>
         </is>
       </c>
     </row>
@@ -7865,7 +8465,11 @@
       </c>
       <c r="K96" t="inlineStr"/>
       <c r="L96" t="inlineStr"/>
-      <c r="M96" t="inlineStr"/>
+      <c r="M96" t="inlineStr">
+        <is>
+          <t>+5411452808580</t>
+        </is>
+      </c>
       <c r="N96" t="inlineStr">
         <is>
           <t>A</t>
@@ -7889,7 +8493,7 @@
       </c>
       <c r="S96" t="inlineStr">
         <is>
-          <t>Mayorista.</t>
+          <t>Mayorista. | otros tel: 5491140245345</t>
         </is>
       </c>
     </row>
@@ -7966,7 +8570,7 @@
       </c>
       <c r="S97" t="inlineStr">
         <is>
-          <t>Bazar, limpieza y hogar.</t>
+          <t>Bazar, limpieza y hogar. | el sitio no publica datos de contacto: buscar por Google Maps o LinkedIn</t>
         </is>
       </c>
     </row>
@@ -8019,7 +8623,11 @@
       </c>
       <c r="K98" t="inlineStr"/>
       <c r="L98" t="inlineStr"/>
-      <c r="M98" t="inlineStr"/>
+      <c r="M98" t="inlineStr">
+        <is>
+          <t>43225700</t>
+        </is>
+      </c>
       <c r="N98" t="inlineStr">
         <is>
           <t>C</t>
@@ -8095,8 +8703,16 @@
         </is>
       </c>
       <c r="K99" t="inlineStr"/>
-      <c r="L99" t="inlineStr"/>
-      <c r="M99" t="inlineStr"/>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>administracion@afadmin.com.ar</t>
+        </is>
+      </c>
+      <c r="M99" t="inlineStr">
+        <is>
+          <t>5491122972298</t>
+        </is>
+      </c>
       <c r="N99" t="inlineStr">
         <is>
           <t>B</t>
@@ -8172,8 +8788,16 @@
         </is>
       </c>
       <c r="K100" t="inlineStr"/>
-      <c r="L100" t="inlineStr"/>
-      <c r="M100" t="inlineStr"/>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>contacto@mgadministracion.com.ar</t>
+        </is>
+      </c>
+      <c r="M100" t="inlineStr">
+        <is>
+          <t>5402236281357</t>
+        </is>
+      </c>
       <c r="N100" t="inlineStr">
         <is>
           <t>C</t>
@@ -8274,7 +8898,7 @@
       </c>
       <c r="S101" t="inlineStr">
         <is>
-          <t>Laboral para empresas: cliente con obligaciones documentales propias.</t>
+          <t>Laboral para empresas: cliente con obligaciones documentales propias. | el sitio no publica datos de contacto: buscar por Google Maps o LinkedIn</t>
         </is>
       </c>
     </row>
@@ -8326,8 +8950,16 @@
         </is>
       </c>
       <c r="K102" t="inlineStr"/>
-      <c r="L102" t="inlineStr"/>
-      <c r="M102" t="inlineStr"/>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t>info@estudioramat.com.ar</t>
+        </is>
+      </c>
+      <c r="M102" t="inlineStr">
+        <is>
+          <t>5491122832784</t>
+        </is>
+      </c>
       <c r="N102" t="inlineStr">
         <is>
           <t>B</t>
@@ -8403,8 +9035,16 @@
         </is>
       </c>
       <c r="K103" t="inlineStr"/>
-      <c r="L103" t="inlineStr"/>
-      <c r="M103" t="inlineStr"/>
+      <c r="L103" t="inlineStr">
+        <is>
+          <t>consultas@asesordeempresas.com.ar</t>
+        </is>
+      </c>
+      <c r="M103" t="inlineStr">
+        <is>
+          <t>541135214859</t>
+        </is>
+      </c>
       <c r="N103" t="inlineStr">
         <is>
           <t>B</t>
@@ -8480,8 +9120,16 @@
         </is>
       </c>
       <c r="K104" t="inlineStr"/>
-      <c r="L104" t="inlineStr"/>
-      <c r="M104" t="inlineStr"/>
+      <c r="L104" t="inlineStr">
+        <is>
+          <t>info@ferrettiabogados.com</t>
+        </is>
+      </c>
+      <c r="M104" t="inlineStr">
+        <is>
+          <t>5491157625152</t>
+        </is>
+      </c>
       <c r="N104" t="inlineStr">
         <is>
           <t>C</t>
@@ -8505,7 +9153,7 @@
       </c>
       <c r="S104" t="inlineStr">
         <is>
-          <t>Laboral, ART, accidentes.</t>
+          <t>Laboral, ART, accidentes. | otros tel: 43310397</t>
         </is>
       </c>
     </row>
@@ -8557,8 +9205,16 @@
         </is>
       </c>
       <c r="K105" t="inlineStr"/>
-      <c r="L105" t="inlineStr"/>
-      <c r="M105" t="inlineStr"/>
+      <c r="L105" t="inlineStr">
+        <is>
+          <t>estudio@grupolegal.com.ar</t>
+        </is>
+      </c>
+      <c r="M105" t="inlineStr">
+        <is>
+          <t>+5491178419797</t>
+        </is>
+      </c>
       <c r="N105" t="inlineStr">
         <is>
           <t>B</t>

</xml_diff>